<commit_message>
feat: Implement report generation for movimientos with Excel export
Co-authored-by: zapata888 <zapata888@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/server/src/templates/formato_movimiento.xlsx
+++ b/server/src/templates/formato_movimiento.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\usuario\Documents\Luisongo\Trayecto III\Aprendiendo Node.js\SIGADBP\server\src\templates\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{01BAB506-4F68-4630-824D-B4DBB301F0B3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4A581317-12B2-49D4-9C02-B88621B5F67F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{9885C519-7CCA-4CFD-8609-2B5C3A63C552}"/>
   </bookViews>
@@ -97,9 +97,6 @@
     <t>ORGANISMO: MERCAL, C.A.</t>
   </si>
   <si>
-    <t>TIPO DE MOVIMIENTO</t>
-  </si>
-  <si>
     <t>DEPENDENCIA ORGANIZATIVA A LA QUE PERTENECE EL BIEN</t>
   </si>
   <si>
@@ -113,6 +110,9 @@
   </si>
   <si>
     <t>FORMATO DE ASIGNACIÓN O MOVIMIENTO DE BIENES</t>
+  </si>
+  <si>
+    <t>TIPO DE INCORPORACIÓN</t>
   </si>
 </sst>
 </file>
@@ -227,10 +227,31 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -255,28 +276,7 @@
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -662,127 +662,127 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A1" s="14"/>
-      <c r="B1" s="15" t="s">
+      <c r="A1" s="9"/>
+      <c r="B1" s="21" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="15"/>
-      <c r="D1" s="5" t="s">
+      <c r="C1" s="21"/>
+      <c r="D1" s="8" t="s">
         <v>14</v>
       </c>
-      <c r="E1" s="5"/>
-      <c r="F1" s="5"/>
-      <c r="G1" s="5"/>
-      <c r="H1" s="5"/>
+      <c r="E1" s="8"/>
+      <c r="F1" s="8"/>
+      <c r="G1" s="8"/>
+      <c r="H1" s="8"/>
       <c r="I1" s="2" t="s">
         <v>2</v>
       </c>
     </row>
     <row r="2" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A2" s="14"/>
-      <c r="B2" s="15" t="s">
+      <c r="A2" s="9"/>
+      <c r="B2" s="21" t="s">
         <v>3</v>
       </c>
-      <c r="C2" s="15"/>
-      <c r="D2" s="5"/>
-      <c r="E2" s="5"/>
-      <c r="F2" s="5"/>
-      <c r="G2" s="5"/>
-      <c r="H2" s="5"/>
+      <c r="C2" s="21"/>
+      <c r="D2" s="8"/>
+      <c r="E2" s="8"/>
+      <c r="F2" s="8"/>
+      <c r="G2" s="8"/>
+      <c r="H2" s="8"/>
       <c r="I2" s="2" t="s">
         <v>13</v>
       </c>
     </row>
     <row r="3" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A3" s="14"/>
-      <c r="B3" s="15" t="s">
+      <c r="A3" s="9"/>
+      <c r="B3" s="21" t="s">
         <v>4</v>
       </c>
-      <c r="C3" s="15"/>
-      <c r="D3" s="5"/>
-      <c r="E3" s="5"/>
-      <c r="F3" s="5"/>
-      <c r="G3" s="5"/>
-      <c r="H3" s="5"/>
+      <c r="C3" s="21"/>
+      <c r="D3" s="8"/>
+      <c r="E3" s="8"/>
+      <c r="F3" s="8"/>
+      <c r="G3" s="8"/>
+      <c r="H3" s="8"/>
       <c r="I3" s="1"/>
     </row>
     <row r="4" spans="1:9" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="5" t="s">
-        <v>25</v>
-      </c>
-      <c r="B4" s="5"/>
-      <c r="C4" s="5"/>
-      <c r="D4" s="5"/>
-      <c r="E4" s="5"/>
-      <c r="F4" s="5"/>
-      <c r="G4" s="5"/>
-      <c r="H4" s="5"/>
-      <c r="I4" s="5"/>
+      <c r="A4" s="8" t="s">
+        <v>24</v>
+      </c>
+      <c r="B4" s="8"/>
+      <c r="C4" s="8"/>
+      <c r="D4" s="8"/>
+      <c r="E4" s="8"/>
+      <c r="F4" s="8"/>
+      <c r="G4" s="8"/>
+      <c r="H4" s="8"/>
+      <c r="I4" s="8"/>
     </row>
     <row r="5" spans="1:9" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="13" t="s">
+      <c r="A5" s="20" t="s">
         <v>19</v>
       </c>
-      <c r="B5" s="13"/>
-      <c r="C5" s="13"/>
-      <c r="D5" s="13"/>
-      <c r="E5" s="13"/>
-      <c r="F5" s="13"/>
-      <c r="G5" s="13"/>
-      <c r="H5" s="13"/>
-      <c r="I5" s="13"/>
+      <c r="B5" s="20"/>
+      <c r="C5" s="20"/>
+      <c r="D5" s="20"/>
+      <c r="E5" s="20"/>
+      <c r="F5" s="20"/>
+      <c r="G5" s="20"/>
+      <c r="H5" s="20"/>
+      <c r="I5" s="20"/>
     </row>
     <row r="6" spans="1:9" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="5" t="s">
+      <c r="A6" s="8" t="s">
+        <v>20</v>
+      </c>
+      <c r="B6" s="8"/>
+      <c r="C6" s="8"/>
+      <c r="D6" s="8"/>
+      <c r="E6" s="8" t="s">
         <v>21</v>
       </c>
-      <c r="B6" s="5"/>
-      <c r="C6" s="5"/>
-      <c r="D6" s="5"/>
-      <c r="E6" s="5" t="s">
+      <c r="F6" s="8"/>
+      <c r="G6" s="8"/>
+      <c r="H6" s="8"/>
+      <c r="I6" s="8"/>
+    </row>
+    <row r="7" spans="1:9" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A7" s="13"/>
+      <c r="B7" s="13"/>
+      <c r="C7" s="13"/>
+      <c r="D7" s="13"/>
+      <c r="E7" s="13"/>
+      <c r="F7" s="13"/>
+      <c r="G7" s="13"/>
+      <c r="H7" s="13"/>
+      <c r="I7" s="13"/>
+    </row>
+    <row r="8" spans="1:9" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A8" s="8" t="s">
         <v>22</v>
       </c>
-      <c r="F6" s="5"/>
-      <c r="G6" s="5"/>
-      <c r="H6" s="5"/>
-      <c r="I6" s="5"/>
-    </row>
-    <row r="7" spans="1:9" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A7" s="6"/>
-      <c r="B7" s="6"/>
-      <c r="C7" s="6"/>
-      <c r="D7" s="6"/>
-      <c r="E7" s="6"/>
-      <c r="F7" s="6"/>
-      <c r="G7" s="6"/>
-      <c r="H7" s="6"/>
-      <c r="I7" s="6"/>
-    </row>
-    <row r="8" spans="1:9" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A8" s="5" t="s">
+      <c r="B8" s="8"/>
+      <c r="C8" s="8"/>
+      <c r="D8" s="8"/>
+      <c r="E8" s="14" t="s">
         <v>23</v>
       </c>
-      <c r="B8" s="5"/>
-      <c r="C8" s="5"/>
-      <c r="D8" s="5"/>
-      <c r="E8" s="7" t="s">
-        <v>24</v>
-      </c>
-      <c r="F8" s="8"/>
-      <c r="G8" s="8"/>
-      <c r="H8" s="8"/>
-      <c r="I8" s="9"/>
+      <c r="F8" s="15"/>
+      <c r="G8" s="15"/>
+      <c r="H8" s="15"/>
+      <c r="I8" s="16"/>
     </row>
     <row r="9" spans="1:9" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A9" s="6"/>
-      <c r="B9" s="6"/>
-      <c r="C9" s="6"/>
-      <c r="D9" s="6"/>
-      <c r="E9" s="10"/>
-      <c r="F9" s="11"/>
-      <c r="G9" s="11"/>
-      <c r="H9" s="11"/>
-      <c r="I9" s="12"/>
+      <c r="A9" s="13"/>
+      <c r="B9" s="13"/>
+      <c r="C9" s="13"/>
+      <c r="D9" s="13"/>
+      <c r="E9" s="17"/>
+      <c r="F9" s="18"/>
+      <c r="G9" s="18"/>
+      <c r="H9" s="18"/>
+      <c r="I9" s="19"/>
     </row>
     <row r="10" spans="1:9" ht="34.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10" s="2" t="s">
@@ -798,7 +798,7 @@
         <v>0</v>
       </c>
       <c r="E10" s="3" t="s">
-        <v>20</v>
+        <v>25</v>
       </c>
       <c r="F10" s="3" t="s">
         <v>6</v>
@@ -1034,82 +1034,69 @@
       <c r="I30" s="4"/>
     </row>
     <row r="31" spans="1:9" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A31" s="16" t="s">
+      <c r="A31" s="5" t="s">
         <v>5</v>
       </c>
-      <c r="B31" s="17"/>
-      <c r="C31" s="17"/>
-      <c r="D31" s="17"/>
-      <c r="E31" s="17"/>
-      <c r="F31" s="17"/>
-      <c r="G31" s="17"/>
-      <c r="H31" s="17"/>
-      <c r="I31" s="18"/>
+      <c r="B31" s="6"/>
+      <c r="C31" s="6"/>
+      <c r="D31" s="6"/>
+      <c r="E31" s="6"/>
+      <c r="F31" s="6"/>
+      <c r="G31" s="6"/>
+      <c r="H31" s="6"/>
+      <c r="I31" s="7"/>
     </row>
     <row r="32" spans="1:9" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A32" s="5" t="s">
+      <c r="A32" s="8" t="s">
         <v>6</v>
       </c>
-      <c r="B32" s="5"/>
-      <c r="C32" s="5"/>
-      <c r="D32" s="5" t="s">
+      <c r="B32" s="8"/>
+      <c r="C32" s="8"/>
+      <c r="D32" s="8" t="s">
         <v>15</v>
       </c>
-      <c r="E32" s="5"/>
-      <c r="F32" s="5" t="s">
+      <c r="E32" s="8"/>
+      <c r="F32" s="8" t="s">
         <v>16</v>
       </c>
-      <c r="G32" s="5"/>
-      <c r="H32" s="5" t="s">
+      <c r="G32" s="8"/>
+      <c r="H32" s="8" t="s">
         <v>17</v>
       </c>
-      <c r="I32" s="5"/>
+      <c r="I32" s="8"/>
     </row>
     <row r="33" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A33" s="14"/>
-      <c r="B33" s="14"/>
-      <c r="C33" s="14"/>
-      <c r="D33" s="14"/>
-      <c r="E33" s="14"/>
-      <c r="F33" s="14"/>
-      <c r="G33" s="14"/>
-      <c r="H33" s="14"/>
-      <c r="I33" s="14"/>
+      <c r="A33" s="9"/>
+      <c r="B33" s="9"/>
+      <c r="C33" s="9"/>
+      <c r="D33" s="9"/>
+      <c r="E33" s="9"/>
+      <c r="F33" s="9"/>
+      <c r="G33" s="9"/>
+      <c r="H33" s="9"/>
+      <c r="I33" s="9"/>
     </row>
     <row r="34" spans="1:9" ht="79.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A34" s="19" t="s">
+      <c r="A34" s="10" t="s">
         <v>18</v>
       </c>
-      <c r="B34" s="21"/>
-      <c r="C34" s="20"/>
-      <c r="D34" s="19" t="s">
+      <c r="B34" s="12"/>
+      <c r="C34" s="11"/>
+      <c r="D34" s="10" t="s">
         <v>18</v>
       </c>
-      <c r="E34" s="20"/>
-      <c r="F34" s="19" t="s">
+      <c r="E34" s="11"/>
+      <c r="F34" s="10" t="s">
         <v>18</v>
       </c>
-      <c r="G34" s="20"/>
-      <c r="H34" s="19" t="s">
+      <c r="G34" s="11"/>
+      <c r="H34" s="10" t="s">
         <v>18</v>
       </c>
-      <c r="I34" s="20"/>
+      <c r="I34" s="11"/>
     </row>
   </sheetData>
   <mergeCells count="28">
-    <mergeCell ref="A31:I31"/>
-    <mergeCell ref="F32:G32"/>
-    <mergeCell ref="F33:G33"/>
-    <mergeCell ref="F34:G34"/>
-    <mergeCell ref="H32:I32"/>
-    <mergeCell ref="H33:I33"/>
-    <mergeCell ref="H34:I34"/>
-    <mergeCell ref="A32:C32"/>
-    <mergeCell ref="A33:C33"/>
-    <mergeCell ref="A34:C34"/>
-    <mergeCell ref="D32:E32"/>
-    <mergeCell ref="D33:E33"/>
-    <mergeCell ref="D34:E34"/>
     <mergeCell ref="A8:D8"/>
     <mergeCell ref="A9:D9"/>
     <mergeCell ref="E8:I8"/>
@@ -1125,6 +1112,19 @@
     <mergeCell ref="B1:C1"/>
     <mergeCell ref="B3:C3"/>
     <mergeCell ref="B2:C2"/>
+    <mergeCell ref="A31:I31"/>
+    <mergeCell ref="F32:G32"/>
+    <mergeCell ref="F33:G33"/>
+    <mergeCell ref="F34:G34"/>
+    <mergeCell ref="H32:I32"/>
+    <mergeCell ref="H33:I33"/>
+    <mergeCell ref="H34:I34"/>
+    <mergeCell ref="A32:C32"/>
+    <mergeCell ref="A33:C33"/>
+    <mergeCell ref="A34:C34"/>
+    <mergeCell ref="D32:E32"/>
+    <mergeCell ref="D33:E33"/>
+    <mergeCell ref="D34:E34"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>

</xml_diff>